<commit_message>
Fixed false positive triggers on COMP output
</commit_message>
<xml_diff>
--- a/DICE-B-Board-BOM.xlsx
+++ b/DICE-B-Board-BOM.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="76">
   <si>
     <t xml:space="preserve">DICE B-Board BOM</t>
   </si>
@@ -138,13 +138,13 @@
     <t xml:space="preserve">C102</t>
   </si>
   <si>
+    <t xml:space="preserve">C23631</t>
+  </si>
+  <si>
     <t xml:space="preserve">1n</t>
   </si>
   <si>
-    <t xml:space="preserve">C23631</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D101,D102,D103,D104,D110,D111,D112,D113,D114</t>
+    <t xml:space="preserve">D101,D102,D103,D104,D110,D111,D112,D113,D114,D117</t>
   </si>
   <si>
     <t xml:space="preserve">C917117</t>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">Connector_PinHeader_2.54mm:PinHeader_1x07_P2.54mm_Vertical</t>
   </si>
   <si>
-    <t xml:space="preserve">Q101,Q102</t>
+    <t xml:space="preserve">Q101,Q102,Q103</t>
   </si>
   <si>
     <t xml:space="preserve">C475630</t>
@@ -195,7 +195,7 @@
     <t xml:space="preserve">Package_TO_SOT_SMD:SOT-23</t>
   </si>
   <si>
-    <t xml:space="preserve">R1</t>
+    <t xml:space="preserve">R1,R134</t>
   </si>
   <si>
     <t xml:space="preserve">C2907373</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">4k7</t>
   </si>
   <si>
-    <t xml:space="preserve">R5,R6,R13,R101,R102,R103,R104,R105,R106,R107,R108,R110,R111,R112,R114,R119</t>
+    <t xml:space="preserve">R5,R6,R13,R101,R102,R103,R104,R105,R106,R107,R108,R110,R111,R112,R114</t>
   </si>
   <si>
     <t xml:space="preserve">C728669</t>
@@ -234,7 +234,7 @@
     <t xml:space="preserve">100k</t>
   </si>
   <si>
-    <t xml:space="preserve">R7,R113,R116,R120</t>
+    <t xml:space="preserve">R7,R113,R116</t>
   </si>
   <si>
     <t xml:space="preserve">C131398</t>
@@ -250,6 +250,15 @@
   </si>
   <si>
     <t xml:space="preserve">10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R119</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C870758</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47k</t>
   </si>
   <si>
     <t xml:space="preserve">R121,R122</t>
@@ -444,7 +453,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -477,19 +486,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -501,7 +514,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -510,11 +523,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -616,9 +629,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>631440</xdr:colOff>
+      <xdr:colOff>631080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>151200</xdr:rowOff>
+      <xdr:rowOff>150840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -632,7 +645,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="209520"/>
-          <a:ext cx="1256400" cy="370440"/>
+          <a:ext cx="1256040" cy="370080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1193,17 +1206,11 @@
       <c r="B11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>13</v>
-      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="2"/>
@@ -1235,18 +1242,17 @@
         <v>1</v>
       </c>
       <c r="D12" s="7"/>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>25</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>24</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="0"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
@@ -1272,7 +1278,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="8" t="s">
@@ -1432,7 +1438,7 @@
         <v>39</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="9" t="s">
@@ -1472,10 +1478,10 @@
         <v>43</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="7"/>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F18" s="7" t="s">
@@ -1515,7 +1521,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="7"/>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F19" s="7" t="s">
@@ -1555,7 +1561,7 @@
         <v>6</v>
       </c>
       <c r="D20" s="7"/>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>51</v>
       </c>
       <c r="F20" s="7" t="s">
@@ -1592,7 +1598,7 @@
         <v>53</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="8" t="s">
@@ -1632,7 +1638,7 @@
         <v>56</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="11" t="s">
@@ -1695,10 +1701,10 @@
         <v>62</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="7"/>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="12" t="s">
         <v>63</v>
       </c>
       <c r="F24" s="7" t="s">
@@ -1735,17 +1741,17 @@
         <v>65</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" s="7"/>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>67</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
@@ -1772,20 +1778,20 @@
         <v>19</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="G26" s="7" t="s">
         <v>71</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>72</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
@@ -1808,26 +1814,47 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F27" s="0"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
-      <c r="M27" s="12"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="12"/>
-      <c r="Q27" s="12"/>
-      <c r="R27" s="12"/>
-      <c r="S27" s="12"/>
-      <c r="T27" s="12"/>
-      <c r="U27" s="12"/>
-      <c r="V27" s="12"/>
-      <c r="W27" s="12"/>
-      <c r="X27" s="12"/>
-      <c r="Y27" s="12"/>
-      <c r="Z27" s="12"/>
+      <c r="A27" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="13"/>
+      <c r="S27" s="13"/>
+      <c r="T27" s="13"/>
+      <c r="U27" s="13"/>
+      <c r="V27" s="13"/>
+      <c r="W27" s="13"/>
+      <c r="X27" s="13"/>
+      <c r="Y27" s="13"/>
+      <c r="Z27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -1847,6 +1874,15 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0"/>
+      <c r="B29" s="0"/>
+      <c r="C29" s="0"/>
+      <c r="D29" s="0"/>
+      <c r="E29" s="0"/>
+      <c r="F29" s="0"/>
+      <c r="G29" s="0"/>
+      <c r="H29" s="0"/>
+      <c r="I29" s="0"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
@@ -1866,6 +1902,15 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0"/>
+      <c r="B30" s="0"/>
+      <c r="C30" s="0"/>
+      <c r="D30" s="0"/>
+      <c r="E30" s="0"/>
+      <c r="F30" s="0"/>
+      <c r="G30" s="0"/>
+      <c r="H30" s="0"/>
+      <c r="I30" s="0"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -1885,6 +1930,15 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0"/>
+      <c r="B31" s="0"/>
+      <c r="C31" s="0"/>
+      <c r="D31" s="0"/>
+      <c r="E31" s="0"/>
+      <c r="F31" s="0"/>
+      <c r="G31" s="0"/>
+      <c r="H31" s="0"/>
+      <c r="I31" s="0"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -1904,6 +1958,15 @@
       <c r="Z31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0"/>
+      <c r="B32" s="0"/>
+      <c r="C32" s="0"/>
+      <c r="D32" s="0"/>
+      <c r="E32" s="0"/>
+      <c r="F32" s="0"/>
+      <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
+      <c r="I32" s="0"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -1923,6 +1986,15 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0"/>
+      <c r="B33" s="0"/>
+      <c r="C33" s="0"/>
+      <c r="D33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="0"/>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -1942,6 +2014,15 @@
       <c r="Z33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
@@ -1961,6 +2042,15 @@
       <c r="Z34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="14"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
@@ -1980,15 +2070,15 @@
       <c r="Z35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13"/>
+      <c r="A36" s="14"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="15"/>
       <c r="F36" s="14"/>
       <c r="G36" s="14"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -2008,15 +2098,15 @@
       <c r="Z36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="15"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="16"/>
       <c r="F37" s="14"/>
       <c r="G37" s="14"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="14"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -2036,15 +2126,15 @@
       <c r="Z37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13"/>
+      <c r="A38" s="14"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="15"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
       <c r="F38" s="14"/>
       <c r="G38" s="14"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -2064,15 +2154,15 @@
       <c r="Z38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13"/>
+      <c r="A39" s="14"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="16"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
       <c r="F39" s="14"/>
       <c r="G39" s="14"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="14"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -2092,15 +2182,15 @@
       <c r="Z39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13"/>
+      <c r="A40" s="14"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="15"/>
       <c r="F40" s="14"/>
       <c r="G40" s="14"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="14"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
@@ -2120,15 +2210,15 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13"/>
+      <c r="A41" s="14"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
       <c r="F41" s="14"/>
       <c r="G41" s="14"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="14"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
@@ -2148,15 +2238,15 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13"/>
+      <c r="A42" s="14"/>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
       <c r="F42" s="14"/>
       <c r="G42" s="14"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -2176,15 +2266,15 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13"/>
+      <c r="A43" s="14"/>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
       <c r="F43" s="14"/>
       <c r="G43" s="14"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -2204,15 +2294,15 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13"/>
+      <c r="A44" s="14"/>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="16"/>
       <c r="F44" s="14"/>
       <c r="G44" s="14"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -2232,15 +2322,15 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13"/>
+      <c r="A45" s="14"/>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
       <c r="F45" s="14"/>
       <c r="G45" s="14"/>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
@@ -2260,15 +2350,15 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13"/>
+      <c r="A46" s="14"/>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
       <c r="F46" s="14"/>
       <c r="G46" s="14"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
@@ -2288,15 +2378,15 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13"/>
+      <c r="A47" s="14"/>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="15"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="16"/>
       <c r="F47" s="14"/>
       <c r="G47" s="14"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
@@ -2316,15 +2406,15 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13"/>
+      <c r="A48" s="14"/>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="15"/>
       <c r="F48" s="14"/>
       <c r="G48" s="14"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
@@ -2344,15 +2434,15 @@
       <c r="Z48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13"/>
+      <c r="A49" s="14"/>
       <c r="B49" s="14"/>
       <c r="C49" s="14"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="15"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="17"/>
       <c r="F49" s="14"/>
       <c r="G49" s="14"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
@@ -2372,15 +2462,15 @@
       <c r="Z49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="13"/>
+      <c r="A50" s="14"/>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
-      <c r="D50" s="13"/>
+      <c r="D50" s="14"/>
       <c r="E50" s="15"/>
       <c r="F50" s="14"/>
       <c r="G50" s="14"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="14"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
@@ -2400,15 +2490,15 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="13"/>
+      <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="14"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
       <c r="F51" s="14"/>
       <c r="G51" s="14"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="13"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
       <c r="L51" s="2"/>
@@ -2428,15 +2518,15 @@
       <c r="Z51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="13"/>
+      <c r="A52" s="14"/>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="15"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="17"/>
       <c r="F52" s="14"/>
       <c r="G52" s="14"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="17"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -2456,15 +2546,15 @@
       <c r="Z52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13"/>
+      <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="17"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
       <c r="F53" s="14"/>
       <c r="G53" s="14"/>
-      <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
       <c r="L53" s="2"/>
@@ -2484,15 +2574,15 @@
       <c r="Z53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="13"/>
+      <c r="A54" s="14"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="14"/>
+      <c r="I54" s="14"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="2"/>
@@ -2512,15 +2602,15 @@
       <c r="Z54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="18"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="13"/>
-      <c r="I55" s="13"/>
+      <c r="A55" s="14"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="19"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
@@ -2540,15 +2630,15 @@
       <c r="Z55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15"/>
-      <c r="B56" s="15"/>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="15"/>
+      <c r="A56" s="16"/>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
+      <c r="H56" s="16"/>
+      <c r="I56" s="16"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2"/>
@@ -2568,15 +2658,15 @@
       <c r="Z56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
+      <c r="A57" s="16"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
       <c r="L57" s="2"/>
@@ -2596,15 +2686,15 @@
       <c r="Z57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="20"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
+      <c r="A58" s="21"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="21"/>
+      <c r="D58" s="21"/>
+      <c r="E58" s="21"/>
+      <c r="F58" s="21"/>
+      <c r="G58" s="21"/>
+      <c r="H58" s="21"/>
+      <c r="I58" s="21"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
       <c r="L58" s="2"/>
@@ -2624,15 +2714,15 @@
       <c r="Z58" s="2"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="21"/>
-      <c r="B59" s="21"/>
-      <c r="C59" s="21"/>
-      <c r="D59" s="21"/>
-      <c r="E59" s="21"/>
-      <c r="F59" s="21"/>
-      <c r="G59" s="21"/>
-      <c r="H59" s="21"/>
-      <c r="I59" s="21"/>
+      <c r="A59" s="22"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="22"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>

</xml_diff>